<commit_message>
chore(weekly-sync): auto-pull through 2026-06-15
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week24.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week24.xlsx
@@ -479,7 +479,7 @@
         <v>49</v>
       </c>
       <c r="F2" t="n">
-        <v>12977</v>
+        <v>12971</v>
       </c>
       <c r="G2" t="n">
         <v>3261.86</v>
@@ -507,7 +507,7 @@
         <v>57</v>
       </c>
       <c r="F3" t="n">
-        <v>12381</v>
+        <v>12378</v>
       </c>
       <c r="G3" t="n">
         <v>3388.14</v>
@@ -535,7 +535,7 @@
         <v>64</v>
       </c>
       <c r="F4" t="n">
-        <v>14216</v>
+        <v>14215</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -678,10 +678,10 @@
         <v>37621</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>7033.05</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -843,7 +843,7 @@
         <v>56</v>
       </c>
       <c r="F15" t="n">
-        <v>2651</v>
+        <v>2649</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -899,7 +899,7 @@
         <v>103</v>
       </c>
       <c r="F17" t="n">
-        <v>16201</v>
+        <v>16200</v>
       </c>
       <c r="G17" t="n">
         <v>2626.27</v>
@@ -927,7 +927,7 @@
         <v>175</v>
       </c>
       <c r="F18" t="n">
-        <v>26596</v>
+        <v>26579</v>
       </c>
       <c r="G18" t="n">
         <v>5250.84</v>
@@ -983,7 +983,7 @@
         <v>219</v>
       </c>
       <c r="F20" t="n">
-        <v>29246</v>
+        <v>29223</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -1039,7 +1039,7 @@
         <v>33</v>
       </c>
       <c r="F22" t="n">
-        <v>7228</v>
+        <v>7225</v>
       </c>
       <c r="G22" t="n">
         <v>4828.82</v>
@@ -1151,7 +1151,7 @@
         <v>303</v>
       </c>
       <c r="F26" t="n">
-        <v>31414</v>
+        <v>31412</v>
       </c>
       <c r="G26" t="n">
         <v>35283.96</v>
@@ -1207,7 +1207,7 @@
         <v>46</v>
       </c>
       <c r="F28" t="n">
-        <v>10787</v>
+        <v>10785</v>
       </c>
       <c r="G28" t="n">
         <v>4489.84</v>
@@ -1263,7 +1263,7 @@
         <v>155</v>
       </c>
       <c r="F30" t="n">
-        <v>10302</v>
+        <v>10298</v>
       </c>
       <c r="G30" t="n">
         <v>6734.76</v>
@@ -1291,7 +1291,7 @@
         <v>307</v>
       </c>
       <c r="F31" t="n">
-        <v>22787</v>
+        <v>22780</v>
       </c>
       <c r="G31" t="n">
         <v>60994.19</v>
@@ -1319,7 +1319,7 @@
         <v>79</v>
       </c>
       <c r="F32" t="n">
-        <v>9755</v>
+        <v>9753</v>
       </c>
       <c r="G32" t="n">
         <v>14105.1</v>
@@ -1347,13 +1347,13 @@
         <v>1241</v>
       </c>
       <c r="F33" t="n">
-        <v>91667</v>
+        <v>91658</v>
       </c>
       <c r="G33" t="n">
         <v>82088.3</v>
       </c>
       <c r="H33" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="34">
@@ -1403,7 +1403,7 @@
         <v>87</v>
       </c>
       <c r="F35" t="n">
-        <v>21885</v>
+        <v>21883</v>
       </c>
       <c r="G35" t="n">
         <v>6438.98</v>
@@ -1487,7 +1487,7 @@
         <v>57</v>
       </c>
       <c r="F38" t="n">
-        <v>6466</v>
+        <v>6464</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
@@ -1711,7 +1711,7 @@
         <v>54</v>
       </c>
       <c r="F46" t="n">
-        <v>6555</v>
+        <v>6552</v>
       </c>
       <c r="G46" t="n">
         <v>0</v>
@@ -1739,7 +1739,7 @@
         <v>206</v>
       </c>
       <c r="F47" t="n">
-        <v>36072</v>
+        <v>36071</v>
       </c>
       <c r="G47" t="n">
         <v>4066.95</v>
@@ -1767,7 +1767,7 @@
         <v>141</v>
       </c>
       <c r="F48" t="n">
-        <v>9097</v>
+        <v>9095</v>
       </c>
       <c r="G48" t="n">
         <v>20351.7</v>
@@ -1823,7 +1823,7 @@
         <v>360</v>
       </c>
       <c r="F50" t="n">
-        <v>56005</v>
+        <v>55980</v>
       </c>
       <c r="G50" t="n">
         <v>28485.6</v>
@@ -1907,7 +1907,7 @@
         <v>968</v>
       </c>
       <c r="F53" t="n">
-        <v>120620</v>
+        <v>120547</v>
       </c>
       <c r="G53" t="n">
         <v>99421.2</v>
@@ -1935,7 +1935,7 @@
         <v>261</v>
       </c>
       <c r="F54" t="n">
-        <v>18409</v>
+        <v>18403</v>
       </c>
       <c r="G54" t="n">
         <v>32535.58</v>
@@ -2131,7 +2131,7 @@
         <v>241</v>
       </c>
       <c r="F61" t="n">
-        <v>46270</v>
+        <v>46269</v>
       </c>
       <c r="G61" t="n">
         <v>18933.07</v>
@@ -2187,7 +2187,7 @@
         <v>47</v>
       </c>
       <c r="F63" t="n">
-        <v>4192</v>
+        <v>4190</v>
       </c>
       <c r="G63" t="n">
         <v>4362.72</v>
@@ -2215,7 +2215,7 @@
         <v>151</v>
       </c>
       <c r="F64" t="n">
-        <v>24171</v>
+        <v>24169</v>
       </c>
       <c r="G64" t="n">
         <v>16623.72</v>
@@ -2271,7 +2271,7 @@
         <v>48</v>
       </c>
       <c r="F66" t="n">
-        <v>3722</v>
+        <v>3721</v>
       </c>
       <c r="G66" t="n">
         <v>30841.52</v>
@@ -2299,7 +2299,7 @@
         <v>52</v>
       </c>
       <c r="F67" t="n">
-        <v>5613</v>
+        <v>5600</v>
       </c>
       <c r="G67" t="n">
         <v>17623.72</v>
@@ -2327,7 +2327,7 @@
         <v>89</v>
       </c>
       <c r="F68" t="n">
-        <v>8978</v>
+        <v>8975</v>
       </c>
       <c r="G68" t="n">
         <v>26469.48</v>
@@ -2411,7 +2411,7 @@
         <v>403</v>
       </c>
       <c r="F71" t="n">
-        <v>75249</v>
+        <v>75238</v>
       </c>
       <c r="G71" t="n">
         <v>2626.27</v>
@@ -2495,7 +2495,7 @@
         <v>57</v>
       </c>
       <c r="F74" t="n">
-        <v>15422</v>
+        <v>15416</v>
       </c>
       <c r="G74" t="n">
         <v>2015.26</v>
@@ -2607,7 +2607,7 @@
         <v>17</v>
       </c>
       <c r="F78" t="n">
-        <v>2439</v>
+        <v>2438</v>
       </c>
       <c r="G78" t="n">
         <v>0</v>
@@ -2691,7 +2691,7 @@
         <v>1082</v>
       </c>
       <c r="F81" t="n">
-        <v>122157</v>
+        <v>122156</v>
       </c>
       <c r="G81" t="n">
         <v>84312.7</v>
@@ -2719,7 +2719,7 @@
         <v>897</v>
       </c>
       <c r="F82" t="n">
-        <v>194770</v>
+        <v>194696</v>
       </c>
       <c r="G82" t="n">
         <v>11219.48</v>
@@ -2775,7 +2775,7 @@
         <v>165</v>
       </c>
       <c r="F84" t="n">
-        <v>14178</v>
+        <v>14176</v>
       </c>
       <c r="G84" t="n">
         <v>9757.639999999999</v>
@@ -2915,7 +2915,7 @@
         <v>103</v>
       </c>
       <c r="F89" t="n">
-        <v>19767</v>
+        <v>19765</v>
       </c>
       <c r="G89" t="n">
         <v>13427.96</v>
@@ -2943,7 +2943,7 @@
         <v>19</v>
       </c>
       <c r="F90" t="n">
-        <v>2152</v>
+        <v>2151</v>
       </c>
       <c r="G90" t="n">
         <v>0</v>
@@ -2971,7 +2971,7 @@
         <v>616</v>
       </c>
       <c r="F91" t="n">
-        <v>66327</v>
+        <v>66270</v>
       </c>
       <c r="G91" t="n">
         <v>21000.84</v>
@@ -3027,7 +3027,7 @@
         <v>92</v>
       </c>
       <c r="F93" t="n">
-        <v>4784</v>
+        <v>4779</v>
       </c>
       <c r="G93" t="n">
         <v>6988.98</v>
@@ -3083,7 +3083,7 @@
         <v>1343</v>
       </c>
       <c r="F95" t="n">
-        <v>116388</v>
+        <v>116363</v>
       </c>
       <c r="G95" t="n">
         <v>119305.08</v>
@@ -3111,13 +3111,13 @@
         <v>677</v>
       </c>
       <c r="F96" t="n">
-        <v>30950</v>
+        <v>30942</v>
       </c>
       <c r="G96" t="n">
-        <v>67787.28</v>
+        <v>74142.36</v>
       </c>
       <c r="H96" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="97">
@@ -3139,7 +3139,7 @@
         <v>259</v>
       </c>
       <c r="F97" t="n">
-        <v>18322</v>
+        <v>18312</v>
       </c>
       <c r="G97" t="n">
         <v>5931.36</v>
@@ -3167,7 +3167,7 @@
         <v>321</v>
       </c>
       <c r="F98" t="n">
-        <v>33375</v>
+        <v>33367</v>
       </c>
       <c r="G98" t="n">
         <v>5930.509999999999</v>
@@ -3223,7 +3223,7 @@
         <v>131</v>
       </c>
       <c r="F100" t="n">
-        <v>13719</v>
+        <v>13714</v>
       </c>
       <c r="G100" t="n">
         <v>13980.5</v>
@@ -3369,7 +3369,7 @@
         <v>11649.15</v>
       </c>
       <c r="H105" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="106">
@@ -3643,7 +3643,7 @@
         <v>102</v>
       </c>
       <c r="F115" t="n">
-        <v>21611</v>
+        <v>21606</v>
       </c>
       <c r="G115" t="n">
         <v>0</v>
@@ -3755,7 +3755,7 @@
         <v>46</v>
       </c>
       <c r="F119" t="n">
-        <v>7781</v>
+        <v>7780</v>
       </c>
       <c r="G119" t="n">
         <v>3981.36</v>
@@ -3783,7 +3783,7 @@
         <v>124</v>
       </c>
       <c r="F120" t="n">
-        <v>29314</v>
+        <v>29303</v>
       </c>
       <c r="G120" t="n">
         <v>4065.24</v>
@@ -4203,7 +4203,7 @@
         <v>111</v>
       </c>
       <c r="F135" t="n">
-        <v>50201</v>
+        <v>50200</v>
       </c>
       <c r="G135" t="n">
         <v>7370.35</v>
@@ -4371,7 +4371,7 @@
         <v>52</v>
       </c>
       <c r="F141" t="n">
-        <v>7843</v>
+        <v>7842</v>
       </c>
       <c r="G141" t="n">
         <v>0</v>
@@ -4483,7 +4483,7 @@
         <v>91</v>
       </c>
       <c r="F145" t="n">
-        <v>18501</v>
+        <v>18500</v>
       </c>
       <c r="G145" t="n">
         <v>1523.73</v>
@@ -4539,7 +4539,7 @@
         <v>2001</v>
       </c>
       <c r="F147" t="n">
-        <v>184410</v>
+        <v>184408</v>
       </c>
       <c r="G147" t="n">
         <v>16096.62</v>
@@ -4710,10 +4710,10 @@
         <v>191806</v>
       </c>
       <c r="G153" t="n">
-        <v>21348.31</v>
+        <v>25415.26</v>
       </c>
       <c r="H153" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="154">
@@ -4791,7 +4791,7 @@
         <v>31</v>
       </c>
       <c r="F156" t="n">
-        <v>3841</v>
+        <v>3840</v>
       </c>
       <c r="G156" t="n">
         <v>5464.41</v>
@@ -5071,7 +5071,7 @@
         <v>283</v>
       </c>
       <c r="F166" t="n">
-        <v>58847</v>
+        <v>58846</v>
       </c>
       <c r="G166" t="n">
         <v>9825.42</v>
@@ -5379,7 +5379,7 @@
         <v>46</v>
       </c>
       <c r="F177" t="n">
-        <v>6977</v>
+        <v>6976</v>
       </c>
       <c r="G177" t="n">
         <v>0</v>
@@ -5631,7 +5631,7 @@
         <v>436</v>
       </c>
       <c r="F186" t="n">
-        <v>93819</v>
+        <v>93817</v>
       </c>
       <c r="G186" t="n">
         <v>6138.97</v>
@@ -5659,7 +5659,7 @@
         <v>306</v>
       </c>
       <c r="F187" t="n">
-        <v>70012</v>
+        <v>70011</v>
       </c>
       <c r="G187" t="n">
         <v>14062.72</v>
@@ -5687,7 +5687,7 @@
         <v>7</v>
       </c>
       <c r="F188" t="n">
-        <v>2954</v>
+        <v>2953</v>
       </c>
       <c r="G188" t="n">
         <v>0</v>
@@ -5799,7 +5799,7 @@
         <v>62</v>
       </c>
       <c r="F192" t="n">
-        <v>8581</v>
+        <v>8580</v>
       </c>
       <c r="G192" t="n">
         <v>0</v>
@@ -6191,13 +6191,13 @@
         <v>332</v>
       </c>
       <c r="F206" t="n">
-        <v>33381</v>
+        <v>33380</v>
       </c>
       <c r="G206" t="n">
-        <v>33850</v>
+        <v>31181.36</v>
       </c>
       <c r="H206" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="207">
@@ -6443,7 +6443,7 @@
         <v>2281</v>
       </c>
       <c r="F215" t="n">
-        <v>346556</v>
+        <v>346553</v>
       </c>
       <c r="G215" t="n">
         <v>9572.029999999999</v>
@@ -6471,7 +6471,7 @@
         <v>330</v>
       </c>
       <c r="F216" t="n">
-        <v>33908</v>
+        <v>33907</v>
       </c>
       <c r="G216" t="n">
         <v>10166.95</v>
@@ -6639,7 +6639,7 @@
         <v>4304</v>
       </c>
       <c r="F222" t="n">
-        <v>591781</v>
+        <v>591778</v>
       </c>
       <c r="G222" t="n">
         <v>24572.88</v>
@@ -6667,7 +6667,7 @@
         <v>559</v>
       </c>
       <c r="F223" t="n">
-        <v>75825</v>
+        <v>75824</v>
       </c>
       <c r="G223" t="n">
         <v>15252.54</v>
@@ -6835,7 +6835,7 @@
         <v>149</v>
       </c>
       <c r="F229" t="n">
-        <v>28742</v>
+        <v>28710</v>
       </c>
       <c r="G229" t="n">
         <v>26692.37</v>
@@ -6863,7 +6863,7 @@
         <v>354</v>
       </c>
       <c r="F230" t="n">
-        <v>38631</v>
+        <v>38620</v>
       </c>
       <c r="G230" t="n">
         <v>12286.44</v>
@@ -6891,7 +6891,7 @@
         <v>48</v>
       </c>
       <c r="F231" t="n">
-        <v>8535</v>
+        <v>8522</v>
       </c>
       <c r="G231" t="n">
         <v>0</v>
@@ -6919,7 +6919,7 @@
         <v>115</v>
       </c>
       <c r="F232" t="n">
-        <v>12085</v>
+        <v>12070</v>
       </c>
       <c r="G232" t="n">
         <v>0</v>
@@ -6947,7 +6947,7 @@
         <v>733</v>
       </c>
       <c r="F233" t="n">
-        <v>27844</v>
+        <v>27836</v>
       </c>
       <c r="G233" t="n">
         <v>41976.25</v>
@@ -6975,7 +6975,7 @@
         <v>498</v>
       </c>
       <c r="F234" t="n">
-        <v>27247</v>
+        <v>27236</v>
       </c>
       <c r="G234" t="n">
         <v>40711.87</v>
@@ -7003,7 +7003,7 @@
         <v>515</v>
       </c>
       <c r="F235" t="n">
-        <v>46811</v>
+        <v>46804</v>
       </c>
       <c r="G235" t="n">
         <v>14066.1</v>
@@ -7031,7 +7031,7 @@
         <v>243</v>
       </c>
       <c r="F236" t="n">
-        <v>33810</v>
+        <v>33804</v>
       </c>
       <c r="G236" t="n">
         <v>16100</v>
@@ -7087,7 +7087,7 @@
         <v>168</v>
       </c>
       <c r="F238" t="n">
-        <v>12391</v>
+        <v>12388</v>
       </c>
       <c r="G238" t="n">
         <v>7033.05</v>
@@ -7115,7 +7115,7 @@
         <v>44</v>
       </c>
       <c r="F239" t="n">
-        <v>4373</v>
+        <v>4369</v>
       </c>
       <c r="G239" t="n">
         <v>0</v>
@@ -7339,7 +7339,7 @@
         <v>588</v>
       </c>
       <c r="F247" t="n">
-        <v>47373</v>
+        <v>47358</v>
       </c>
       <c r="G247" t="n">
         <v>68492.49000000001</v>
@@ -7423,7 +7423,7 @@
         <v>104</v>
       </c>
       <c r="F250" t="n">
-        <v>9986</v>
+        <v>9981</v>
       </c>
       <c r="G250" t="n">
         <v>5082.21</v>
@@ -7563,7 +7563,7 @@
         <v>18</v>
       </c>
       <c r="F255" t="n">
-        <v>4606</v>
+        <v>4602</v>
       </c>
       <c r="G255" t="n">
         <v>0</v>
@@ -7647,7 +7647,7 @@
         <v>59</v>
       </c>
       <c r="F258" t="n">
-        <v>15767</v>
+        <v>15763</v>
       </c>
       <c r="G258" t="n">
         <v>3879.71</v>
@@ -7703,7 +7703,7 @@
         <v>99</v>
       </c>
       <c r="F260" t="n">
-        <v>16593</v>
+        <v>16592</v>
       </c>
       <c r="G260" t="n">
         <v>5503.4</v>
@@ -7871,7 +7871,7 @@
         <v>26</v>
       </c>
       <c r="F266" t="n">
-        <v>5519</v>
+        <v>5518</v>
       </c>
       <c r="G266" t="n">
         <v>2075.42</v>
@@ -7983,7 +7983,7 @@
         <v>378</v>
       </c>
       <c r="F270" t="n">
-        <v>59463</v>
+        <v>59457</v>
       </c>
       <c r="G270" t="n">
         <v>16940.69</v>
@@ -8067,7 +8067,7 @@
         <v>96</v>
       </c>
       <c r="F273" t="n">
-        <v>26997</v>
+        <v>26996</v>
       </c>
       <c r="G273" t="n">
         <v>12200</v>
@@ -8095,7 +8095,7 @@
         <v>23</v>
       </c>
       <c r="F274" t="n">
-        <v>2651</v>
+        <v>2650</v>
       </c>
       <c r="G274" t="n">
         <v>0</v>
@@ -8123,7 +8123,7 @@
         <v>236</v>
       </c>
       <c r="F275" t="n">
-        <v>38831</v>
+        <v>38810</v>
       </c>
       <c r="G275" t="n">
         <v>5379.66</v>
@@ -8151,7 +8151,7 @@
         <v>53</v>
       </c>
       <c r="F276" t="n">
-        <v>10764</v>
+        <v>10763</v>
       </c>
       <c r="G276" t="n">
         <v>1007.63</v>
@@ -8179,7 +8179,7 @@
         <v>64</v>
       </c>
       <c r="F277" t="n">
-        <v>15728</v>
+        <v>15726</v>
       </c>
       <c r="G277" t="n">
         <v>5038.15</v>
@@ -8207,7 +8207,7 @@
         <v>349</v>
       </c>
       <c r="F278" t="n">
-        <v>49060</v>
+        <v>49054</v>
       </c>
       <c r="G278" t="n">
         <v>24053.33</v>
@@ -8235,7 +8235,7 @@
         <v>94</v>
       </c>
       <c r="F279" t="n">
-        <v>9747</v>
+        <v>9743</v>
       </c>
       <c r="G279" t="n">
         <v>0</v>
@@ -8263,7 +8263,7 @@
         <v>91</v>
       </c>
       <c r="F280" t="n">
-        <v>12394</v>
+        <v>12386</v>
       </c>
       <c r="G280" t="n">
         <v>13555.07</v>
@@ -8291,7 +8291,7 @@
         <v>232</v>
       </c>
       <c r="F281" t="n">
-        <v>39810</v>
+        <v>39782</v>
       </c>
       <c r="G281" t="n">
         <v>14136.44</v>
@@ -8319,7 +8319,7 @@
         <v>896</v>
       </c>
       <c r="F282" t="n">
-        <v>133754</v>
+        <v>133745</v>
       </c>
       <c r="G282" t="n">
         <v>43289.07</v>
@@ -8347,7 +8347,7 @@
         <v>49</v>
       </c>
       <c r="F283" t="n">
-        <v>4007</v>
+        <v>4002</v>
       </c>
       <c r="G283" t="n">
         <v>1395.75</v>
@@ -8375,7 +8375,7 @@
         <v>99</v>
       </c>
       <c r="F284" t="n">
-        <v>19730</v>
+        <v>19729</v>
       </c>
       <c r="G284" t="n">
         <v>2880.51</v>
@@ -8403,7 +8403,7 @@
         <v>766</v>
       </c>
       <c r="F285" t="n">
-        <v>260664</v>
+        <v>260648</v>
       </c>
       <c r="G285" t="n">
         <v>5122.87</v>
@@ -8459,7 +8459,7 @@
         <v>686</v>
       </c>
       <c r="F287" t="n">
-        <v>170460</v>
+        <v>170451</v>
       </c>
       <c r="G287" t="n">
         <v>8171.18</v>
@@ -8683,7 +8683,7 @@
         <v>81</v>
       </c>
       <c r="F295" t="n">
-        <v>10376</v>
+        <v>10372</v>
       </c>
       <c r="G295" t="n">
         <v>15760.17</v>
@@ -9019,7 +9019,7 @@
         <v>66</v>
       </c>
       <c r="F307" t="n">
-        <v>10151</v>
+        <v>10149</v>
       </c>
       <c r="G307" t="n">
         <v>7880.51</v>
@@ -9103,13 +9103,13 @@
         <v>393</v>
       </c>
       <c r="F310" t="n">
-        <v>45464</v>
+        <v>45462</v>
       </c>
       <c r="G310" t="n">
         <v>35584.75</v>
       </c>
       <c r="H310" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="311">
@@ -9131,13 +9131,13 @@
         <v>851</v>
       </c>
       <c r="F311" t="n">
-        <v>83500</v>
+        <v>83491</v>
       </c>
       <c r="G311" t="n">
-        <v>36126.26</v>
+        <v>38455.92</v>
       </c>
       <c r="H311" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="312">
@@ -9243,7 +9243,7 @@
         <v>13</v>
       </c>
       <c r="F315" t="n">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="G315" t="n">
         <v>0</v>
@@ -9383,7 +9383,7 @@
         <v>31</v>
       </c>
       <c r="F320" t="n">
-        <v>3303</v>
+        <v>3300</v>
       </c>
       <c r="G320" t="n">
         <v>2201.7</v>
@@ -9439,7 +9439,7 @@
         <v>57</v>
       </c>
       <c r="F322" t="n">
-        <v>8493</v>
+        <v>8490</v>
       </c>
       <c r="G322" t="n">
         <v>3219.49</v>
@@ -9523,7 +9523,7 @@
         <v>27</v>
       </c>
       <c r="F325" t="n">
-        <v>3821</v>
+        <v>3820</v>
       </c>
       <c r="G325" t="n">
         <v>10970.36</v>
@@ -9551,7 +9551,7 @@
         <v>283</v>
       </c>
       <c r="F326" t="n">
-        <v>23897</v>
+        <v>23893</v>
       </c>
       <c r="G326" t="n">
         <v>9743.219999999999</v>
@@ -9663,7 +9663,7 @@
         <v>85</v>
       </c>
       <c r="F330" t="n">
-        <v>17915</v>
+        <v>17912</v>
       </c>
       <c r="G330" t="n">
         <v>9319.49</v>
@@ -9691,7 +9691,7 @@
         <v>229</v>
       </c>
       <c r="F331" t="n">
-        <v>27188</v>
+        <v>27187</v>
       </c>
       <c r="G331" t="n">
         <v>11094.9</v>
@@ -9915,7 +9915,7 @@
         <v>13</v>
       </c>
       <c r="F339" t="n">
-        <v>2381</v>
+        <v>2380</v>
       </c>
       <c r="G339" t="n">
         <v>3261.86</v>
@@ -10195,7 +10195,7 @@
         <v>262</v>
       </c>
       <c r="F349" t="n">
-        <v>22869</v>
+        <v>22868</v>
       </c>
       <c r="G349" t="n">
         <v>6609.360000000001</v>
@@ -10363,7 +10363,7 @@
         <v>9</v>
       </c>
       <c r="F355" t="n">
-        <v>1355</v>
+        <v>1354</v>
       </c>
       <c r="G355" t="n">
         <v>0</v>
@@ -10419,7 +10419,7 @@
         <v>114</v>
       </c>
       <c r="F357" t="n">
-        <v>17817</v>
+        <v>17816</v>
       </c>
       <c r="G357" t="n">
         <v>3942.48</v>
@@ -10559,7 +10559,7 @@
         <v>22</v>
       </c>
       <c r="F362" t="n">
-        <v>2334</v>
+        <v>2333</v>
       </c>
       <c r="G362" t="n">
         <v>0</v>
@@ -10699,7 +10699,7 @@
         <v>94</v>
       </c>
       <c r="F367" t="n">
-        <v>11816</v>
+        <v>11814</v>
       </c>
       <c r="G367" t="n">
         <v>1397.46</v>
@@ -10727,7 +10727,7 @@
         <v>223</v>
       </c>
       <c r="F368" t="n">
-        <v>21089</v>
+        <v>21085</v>
       </c>
       <c r="G368" t="n">
         <v>0</v>
@@ -11063,7 +11063,7 @@
         <v>183</v>
       </c>
       <c r="F380" t="n">
-        <v>17024</v>
+        <v>17023</v>
       </c>
       <c r="G380" t="n">
         <v>42324.59</v>
@@ -11259,7 +11259,7 @@
         <v>13</v>
       </c>
       <c r="F387" t="n">
-        <v>2839</v>
+        <v>2838</v>
       </c>
       <c r="G387" t="n">
         <v>0</v>
@@ -11293,7 +11293,7 @@
         <v>5641.96</v>
       </c>
       <c r="H388" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="389">
@@ -11315,7 +11315,7 @@
         <v>455</v>
       </c>
       <c r="F389" t="n">
-        <v>45906</v>
+        <v>45904</v>
       </c>
       <c r="G389" t="n">
         <v>19357.62</v>
@@ -11343,7 +11343,7 @@
         <v>787</v>
       </c>
       <c r="F390" t="n">
-        <v>60191</v>
+        <v>60186</v>
       </c>
       <c r="G390" t="n">
         <v>12286.44</v>
@@ -11455,7 +11455,7 @@
         <v>117</v>
       </c>
       <c r="F394" t="n">
-        <v>19671</v>
+        <v>19669</v>
       </c>
       <c r="G394" t="n">
         <v>2117.8</v>
@@ -11483,7 +11483,7 @@
         <v>243</v>
       </c>
       <c r="F395" t="n">
-        <v>28228</v>
+        <v>28225</v>
       </c>
       <c r="G395" t="n">
         <v>0</v>
@@ -11539,7 +11539,7 @@
         <v>55</v>
       </c>
       <c r="F397" t="n">
-        <v>10311</v>
+        <v>10310</v>
       </c>
       <c r="G397" t="n">
         <v>0</v>
@@ -11651,7 +11651,7 @@
         <v>91</v>
       </c>
       <c r="F401" t="n">
-        <v>11108</v>
+        <v>11106</v>
       </c>
       <c r="G401" t="n">
         <v>4236.44</v>
@@ -12071,7 +12071,7 @@
         <v>349</v>
       </c>
       <c r="F416" t="n">
-        <v>32180</v>
+        <v>32177</v>
       </c>
       <c r="G416" t="n">
         <v>24494.5</v>
@@ -12155,7 +12155,7 @@
         <v>138</v>
       </c>
       <c r="F419" t="n">
-        <v>24366</v>
+        <v>24364</v>
       </c>
       <c r="G419" t="n">
         <v>11861.02</v>
@@ -12183,7 +12183,7 @@
         <v>163</v>
       </c>
       <c r="F420" t="n">
-        <v>23711</v>
+        <v>23704</v>
       </c>
       <c r="G420" t="n">
         <v>15246.62</v>
@@ -12211,7 +12211,7 @@
         <v>186</v>
       </c>
       <c r="F421" t="n">
-        <v>34716</v>
+        <v>34715</v>
       </c>
       <c r="G421" t="n">
         <v>13508.37</v>
@@ -12239,7 +12239,7 @@
         <v>56</v>
       </c>
       <c r="F422" t="n">
-        <v>10464</v>
+        <v>10463</v>
       </c>
       <c r="G422" t="n">
         <v>0</v>
@@ -12323,7 +12323,7 @@
         <v>162</v>
       </c>
       <c r="F425" t="n">
-        <v>44755</v>
+        <v>44750</v>
       </c>
       <c r="G425" t="n">
         <v>3388.14</v>
@@ -12379,7 +12379,7 @@
         <v>72</v>
       </c>
       <c r="F427" t="n">
-        <v>14163</v>
+        <v>14162</v>
       </c>
       <c r="G427" t="n">
         <v>9148.309999999999</v>
@@ -12407,7 +12407,7 @@
         <v>89</v>
       </c>
       <c r="F428" t="n">
-        <v>16363</v>
+        <v>16360</v>
       </c>
       <c r="G428" t="n">
         <v>0</v>
@@ -12435,7 +12435,7 @@
         <v>14</v>
       </c>
       <c r="F429" t="n">
-        <v>8309</v>
+        <v>8308</v>
       </c>
       <c r="G429" t="n">
         <v>0</v>
@@ -12463,7 +12463,7 @@
         <v>40</v>
       </c>
       <c r="F430" t="n">
-        <v>14167</v>
+        <v>14166</v>
       </c>
       <c r="G430" t="n">
         <v>0</v>
@@ -12659,7 +12659,7 @@
         <v>57</v>
       </c>
       <c r="F437" t="n">
-        <v>10566</v>
+        <v>10565</v>
       </c>
       <c r="G437" t="n">
         <v>7370.34</v>
@@ -12687,7 +12687,7 @@
         <v>7</v>
       </c>
       <c r="F438" t="n">
-        <v>959</v>
+        <v>956</v>
       </c>
       <c r="G438" t="n">
         <v>0</v>
@@ -12771,7 +12771,7 @@
         <v>99</v>
       </c>
       <c r="F441" t="n">
-        <v>28591</v>
+        <v>28590</v>
       </c>
       <c r="G441" t="n">
         <v>3195.73</v>
@@ -12799,7 +12799,7 @@
         <v>44</v>
       </c>
       <c r="F442" t="n">
-        <v>19186</v>
+        <v>19182</v>
       </c>
       <c r="G442" t="n">
         <v>4616.950000000001</v>
@@ -13026,10 +13026,10 @@
         <v>82055</v>
       </c>
       <c r="G6" t="n">
-        <v>16940.7</v>
+        <v>18634.77</v>
       </c>
       <c r="H6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
@@ -13325,10 +13325,10 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>460.16</v>
+        <v>458.15</v>
       </c>
       <c r="E17" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F17" t="n">
         <v>35261</v>
@@ -13530,10 +13530,10 @@
         <v>20885</v>
       </c>
       <c r="G24" t="n">
-        <v>9149.16</v>
+        <v>10843.23</v>
       </c>
       <c r="H24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
@@ -13605,13 +13605,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>4479.12</v>
+        <v>4476.28</v>
       </c>
       <c r="E27" t="n">
-        <v>1787</v>
+        <v>1785</v>
       </c>
       <c r="F27" t="n">
-        <v>446787</v>
+        <v>446785</v>
       </c>
       <c r="G27" t="n">
         <v>5931.36</v>
@@ -13807,7 +13807,7 @@
         <v>661</v>
       </c>
       <c r="F34" t="n">
-        <v>157623</v>
+        <v>157621</v>
       </c>
       <c r="G34" t="n">
         <v>2329.66</v>
@@ -13866,10 +13866,10 @@
         <v>19673</v>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>3982.2</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -13941,13 +13941,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>8063.92</v>
+        <v>8058.63</v>
       </c>
       <c r="E39" t="n">
-        <v>4401</v>
+        <v>4396</v>
       </c>
       <c r="F39" t="n">
-        <v>1175048</v>
+        <v>1175042</v>
       </c>
       <c r="G39" t="n">
         <v>13048.3</v>

</xml_diff>